<commit_message>
Correct Vitalabs: NSF scope is packaging only, capsules sourced from others
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pAYVPcDWTLeuLdwVsKmmQ
</commit_message>
<xml_diff>
--- a/suppliers_us/Aldera_capsule_price_requests_2026-10-29.xlsx
+++ b/suppliers_us/Aldera_capsule_price_requests_2026-10-29.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Есть (капсулы)</t>
+          <t>Есть, но только как Packaging Facility (фасовка), не производство</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>250+ готовых формул; ещё и фасуют в пакетики. Спросить магний бисглицинат и ашваганду россыпью</t>
+          <t>250+ готовых формул; ещё и фасуют в пакетики. Спросить магний бисглицинат и ашваганду россыпью | ПОПРАВКА 29.10: в реестре NSF Vitalabs записан как Packaging Facility (фасовка и маркировка), без инкапсуляции; капсулы закупают у других (коды bulk-источников HS-MBG01, HS-CO01, см. QUOTES_RAW 02.10). Страна происхождения капсул неизвестна.</t>
         </is>
       </c>
     </row>

</xml_diff>